<commit_message>
Document and formalize 7 reproducible scheduler failure cases using default bug template
Agent-Logs-Url: https://github.com/ArnavBallinCode/TimetableIIITDWD2/sessions/8ed59493-682b-4716-9252-3154ad830898

Co-authored-by: ArnavBallinCode <172006421+ArnavBallinCode@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/test_data/mock_output.xlsx
+++ b/tests/test_data/mock_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestSheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TestSheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,24 +417,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>09:30-11:00</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>11:00-12:30</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
@@ -456,7 +444,7 @@
       <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
@@ -466,7 +454,7 @@
       <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
@@ -476,7 +464,7 @@
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -486,7 +474,7 @@
       <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>

</xml_diff>

<commit_message>
ci: add initial github actions workflow
Agent-Logs-Url: https://github.com/ArnavBallinCode/TimetableIIITDWD2/sessions/3b931196-a619-46e2-bc37-14f540548a9e

Co-authored-by: ArnavBallinCode <172006421+ArnavBallinCode@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/test_data/mock_output.xlsx
+++ b/tests/test_data/mock_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestSheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TestSheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,24 +417,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>09:30-11:00</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>11:00-12:30</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
@@ -456,7 +444,7 @@
       <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
@@ -466,7 +454,7 @@
       <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
@@ -476,7 +464,7 @@
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
@@ -486,7 +474,7 @@
       <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>

</xml_diff>

<commit_message>
chore: address code review feedback and stabilize assertions
Agent-Logs-Url: https://github.com/ArnavBallinCode/TimetableIIITDWD2/sessions/a1f1dda0-b7c3-4231-97e6-59906b054bfe

Co-authored-by: ArnavBallinCode <172006421+ArnavBallinCode@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/test_data/mock_output.xlsx
+++ b/tests/test_data/mock_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestSheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TestSheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,24 +417,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>09:30-11:00</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>11:00-12:30</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Monday</t>
         </is>
@@ -456,37 +444,53 @@
       <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Tuesday</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CS102 (R101)</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Wednesday</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Elective_1</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Thursday</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Elective_1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CS102 (R101)</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Friday</t>
         </is>

</xml_diff>